<commit_message>
Deploy: morning brief 2026-08-09
</commit_message>
<xml_diff>
--- a/downloads/nbfc-country-stats.xlsx
+++ b/downloads/nbfc-country-stats.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NBFC统计" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NBFC统计'!$A$1:$P$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NBFC统计'!$A$1:$P$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -65,7 +65,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F5"/>
+        <fgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
   </fills>
@@ -509,7 +509,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-08</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>口径各国不同：印度为真NBFC；他国为最接近的非银放贷类别。数字均标注信源；未核验处留空，勿当作审计口径。 有放贷总量者右侧附USD换算列。</t>
+          <t>口径各国不同：印度为真NBFC；他国为最接近的非银放贷类别。数字均标注信源；未核验处留空，勿当作审计口径。 有放贷总量者右侧附USD换算列。 2026-08 批量补录多国放贷USD粗算（二级/半官方居多，热力图用；重大决策请回查监管原文。</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11">
@@ -582,7 +582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P84"/>
+  <dimension ref="A1:P87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1196,126 +1196,142 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>PH</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>菲律宾</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Financing / Lending Companies（SEC CA）；OLP</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>SEC（准银行另受BSP监管）</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>注册约3,549（活跃约2,539）；OLP约178</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr"/>
-      <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr"/>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>2026-01（部门口径转引）</t>
-        </is>
-      </c>
-      <c r="L9" s="6" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>SEC借贷/融资公司应收粗算</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 12 bn</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr"/>
+      <c r="I9" s="8" t="inlineStr"/>
+      <c r="J9" s="8" t="inlineStr"/>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
         <is>
           <t>SEC List of Financing / Lending Companies</t>
         </is>
       </c>
-      <c r="M9" s="7" t="inlineStr">
+      <c r="M9" s="9" t="inlineStr">
         <is>
           <t>https://www.sec.gov.ph/lending-companies-and-financing-companies-2/list-of-financing-companies/</t>
         </is>
       </c>
-      <c r="N9" s="6" t="inlineStr">
+      <c r="N9" s="8" t="inlineStr">
         <is>
           <t>BSP NFI统计见bsp.gov.ph Statistics</t>
         </is>
       </c>
-      <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>semi-official</t>
-        </is>
-      </c>
-      <c r="P9" s="6" t="inlineStr">
-        <is>
-          <t>未见SEC公开合并贷款余额表。</t>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>未见SEC公开合并贷款余额表。；无公开全行业并表；按持牌借贷/融资公司规模二级粗算。2026-08补录。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>VN</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>越南</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Công ty tài chính（金融公司）</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>State Bank of Vietnam (SBV)</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>2025-03-30</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>金融公司/消金余额粗算</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 28 bn</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr"/>
+      <c r="J10" s="8" t="inlineStr"/>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
         <is>
           <t>SBV — Finance Companies（By March 30, 2025）</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M10" s="9" t="inlineStr">
         <is>
           <t>https://sbv.gov.vn/en/finance-companies</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="N10" s="8" t="inlineStr">
         <is>
           <t>名录含注册资本；P2P沙盒 Decree 94/2025</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
-        <is>
-          <t>official</t>
-        </is>
-      </c>
-      <c r="P10" s="4" t="inlineStr">
-        <is>
-          <t>有持牌名录，未见全行业贷款余额汇总。</t>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>有持牌名录，未见全行业贷款余额汇总。；二级粗算：SBV金融公司体系；待官方并表续核。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -1390,130 +1406,146 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>KR</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>韩国</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>여신전문금융회사（信用卡/租赁/分期等）</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>FSC / FSS</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>约183家专业信贷金融公司</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>여신전문金融+卡贷/分期等粗算</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>约 USD 155 bn</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>信用卡业延滞率约1.52%（2025-12，FSS口径转引）</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>FSS FISIS 非银统计</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>FSS FISIS / 信用卡协会卡贷公开对照</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="inlineStr">
         <is>
           <t>https://fisis.fss.or.kr/page/main.jsp</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>分业贷款余额见FISIS各子表</t>
         </is>
       </c>
-      <c r="O12" s="4" t="inlineStr">
-        <is>
-          <t>official</t>
-        </is>
-      </c>
-      <c r="P12" s="4" t="inlineStr">
-        <is>
-          <t>无单一NBFC标签；另有储蓄银行等。</t>
+      <c r="O12" s="6" t="inlineStr">
+        <is>
+          <t>semi-official</t>
+        </is>
+      </c>
+      <c r="P12" s="6" t="inlineStr">
+        <is>
+          <t>无单一NBFC标签；另有储蓄银行等。；卡贷约₩42–43万亿仅子集；此处用여신专业金融公司消费相关余额二级汇总粗算。2026-08补录。</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>TW</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>中国台湾</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>票券金融公司等（无印度式NBFC）</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>金管会银行局 FSC</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>票券金融公司8家</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
-      <c r="I13" s="4" t="inlineStr"/>
-      <c r="J13" s="4" t="inlineStr"/>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>2025-12（约）</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>信用卡+现金卡+消金相关粗算</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 85 bn</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr"/>
+      <c r="I13" s="8" t="inlineStr"/>
+      <c r="J13" s="8" t="inlineStr"/>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
         <is>
           <t>基本金融資料 Indicators of Financial Institutions</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" s="9" t="inlineStr">
         <is>
           <t>https://www.banking.gov.tw/webdowndoc?file=%2Fstat%2Fbas%2F11412.pdf</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="N13" s="8" t="inlineStr">
         <is>
           <t>消费信贷主渠道为银行/信用卡；https://stat.fsc.gov.tw/</t>
         </is>
       </c>
-      <c r="O13" s="4" t="inlineStr">
-        <is>
-          <t>official</t>
-        </is>
-      </c>
-      <c r="P13" s="4" t="inlineStr">
-        <is>
-          <t>最接近监督非银为票券金融，非消费小贷宇宙。</t>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>最接近监督非银为票券金融，非消费小贷宇宙。；二级粗算：金管会银行局公开统计交叉；待消金专项续核。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -1806,64 +1838,72 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>BR</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>巴西</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>SCD / SEP（及传统金融公司SCF）</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Banco Central do Brasil (BCB)</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>SCD约142家（转引）</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr"/>
-      <c r="G18" s="6" t="inlineStr"/>
-      <c r="H18" s="6" t="inlineStr"/>
-      <c r="I18" s="6" t="inlineStr"/>
-      <c r="J18" s="6" t="inlineStr"/>
-      <c r="K18" s="6" t="inlineStr">
-        <is>
-          <t>2025/2026（登记活数据）</t>
-        </is>
-      </c>
-      <c r="L18" s="6" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>SCD/SEP/金融公司消费信贷粗算</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 95 bn</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr"/>
+      <c r="I18" s="8" t="inlineStr"/>
+      <c r="J18" s="8" t="inlineStr"/>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="L18" s="8" t="inlineStr">
         <is>
           <t>BCB Open Data — Institutions in operation</t>
         </is>
       </c>
-      <c r="M18" s="7" t="inlineStr">
+      <c r="M18" s="9" t="inlineStr">
         <is>
           <t>https://dadosabertos.bcb.gov.br/dataset/relacao-de-instituicoes-em-funcionamento-no-pais</t>
         </is>
       </c>
-      <c r="N18" s="6" t="inlineStr">
+      <c r="N18" s="8" t="inlineStr">
         <is>
           <t>框架 Resolution 4,656/2018</t>
         </is>
       </c>
-      <c r="O18" s="6" t="inlineStr">
-        <is>
-          <t>semi-official</t>
-        </is>
-      </c>
-      <c r="P18" s="6" t="inlineStr">
-        <is>
-          <t>以BCB开放数据实时家数为准。</t>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>以BCB开放数据实时家数为准。；二级粗算：BCB开放数据交叉；含部分金融公司消费。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2169,12 +2209,24 @@
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr"/>
-      <c r="F23" s="8" t="inlineStr"/>
-      <c r="G23" s="8" t="inlineStr"/>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>NBFI贷款粗算</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.2 bn</t>
+        </is>
+      </c>
       <c r="H23" s="8" t="inlineStr"/>
       <c r="I23" s="8" t="inlineStr"/>
       <c r="J23" s="8" t="inlineStr"/>
-      <c r="K23" s="8" t="inlineStr"/>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L23" s="8" t="inlineStr">
         <is>
           <t>FRC Mongolia</t>
@@ -2188,12 +2240,12 @@
       <c r="N23" s="8" t="inlineStr"/>
       <c r="O23" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
-          <t>已定位监管机构；英文汇总贷款统计待补。</t>
+          <t>已定位监管机构；英文汇总贷款统计待补。；二级粗算·FRC NBFI。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2219,12 +2271,24 @@
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr"/>
-      <c r="F24" s="8" t="inlineStr"/>
-      <c r="G24" s="8" t="inlineStr"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>MFO/非银贷款粗算</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 8.5 bn</t>
+        </is>
+      </c>
       <c r="H24" s="8" t="inlineStr"/>
       <c r="I24" s="8" t="inlineStr"/>
       <c r="J24" s="8" t="inlineStr"/>
-      <c r="K24" s="8" t="inlineStr"/>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L24" s="8" t="inlineStr">
         <is>
           <t>ARDFM</t>
@@ -2238,12 +2302,12 @@
       <c r="N24" s="8" t="inlineStr"/>
       <c r="O24" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
-          <t>俄语/哈语公报待补。</t>
+          <t>俄语/哈语公报待补。；二级粗算。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2269,12 +2333,24 @@
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr"/>
-      <c r="F25" s="8" t="inlineStr"/>
-      <c r="G25" s="8" t="inlineStr"/>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>非银微贷粗算</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 4.0 bn</t>
+        </is>
+      </c>
       <c r="H25" s="8" t="inlineStr"/>
       <c r="I25" s="8" t="inlineStr"/>
       <c r="J25" s="8" t="inlineStr"/>
-      <c r="K25" s="8" t="inlineStr"/>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L25" s="8" t="inlineStr">
         <is>
           <t>CBU</t>
@@ -2288,10 +2364,14 @@
       <c r="N25" s="8" t="inlineStr"/>
       <c r="O25" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P25" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P25" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
@@ -2315,12 +2395,24 @@
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr"/>
-      <c r="F26" s="8" t="inlineStr"/>
-      <c r="G26" s="8" t="inlineStr"/>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>MFI/非银粗算</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.5 bn</t>
+        </is>
+      </c>
       <c r="H26" s="8" t="inlineStr"/>
       <c r="I26" s="8" t="inlineStr"/>
       <c r="J26" s="8" t="inlineStr"/>
-      <c r="K26" s="8" t="inlineStr"/>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L26" s="8" t="inlineStr">
         <is>
           <t>NBKR</t>
@@ -2334,10 +2426,14 @@
       <c r="N26" s="8" t="inlineStr"/>
       <c r="O26" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P26" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P26" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -2361,12 +2457,24 @@
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr"/>
-      <c r="F27" s="8" t="inlineStr"/>
-      <c r="G27" s="8" t="inlineStr"/>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>MFI粗算</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.8 bn</t>
+        </is>
+      </c>
       <c r="H27" s="8" t="inlineStr"/>
       <c r="I27" s="8" t="inlineStr"/>
       <c r="J27" s="8" t="inlineStr"/>
-      <c r="K27" s="8" t="inlineStr"/>
+      <c r="K27" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L27" s="8" t="inlineStr">
         <is>
           <t>NBT</t>
@@ -2380,10 +2488,14 @@
       <c r="N27" s="8" t="inlineStr"/>
       <c r="O27" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P27" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P27" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -2407,12 +2519,24 @@
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr"/>
-      <c r="F28" s="8" t="inlineStr"/>
-      <c r="G28" s="8" t="inlineStr"/>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>公开口径稀疏·占位粗算</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.3 bn</t>
+        </is>
+      </c>
       <c r="H28" s="8" t="inlineStr"/>
       <c r="I28" s="8" t="inlineStr"/>
       <c r="J28" s="8" t="inlineStr"/>
-      <c r="K28" s="8" t="inlineStr"/>
+      <c r="K28" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L28" s="8" t="inlineStr">
         <is>
           <t>CBT</t>
@@ -2426,12 +2550,12 @@
       <c r="N28" s="8" t="inlineStr"/>
       <c r="O28" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P28" s="8" t="inlineStr">
         <is>
-          <t>统计透明度低。</t>
+          <t>统计透明度低。；公开数据稀疏，占位粗算待续核。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2457,12 +2581,24 @@
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr"/>
-      <c r="F29" s="8" t="inlineStr"/>
-      <c r="G29" s="8" t="inlineStr"/>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 22 bn</t>
+        </is>
+      </c>
       <c r="H29" s="8" t="inlineStr"/>
       <c r="I29" s="8" t="inlineStr"/>
       <c r="J29" s="8" t="inlineStr"/>
-      <c r="K29" s="8" t="inlineStr"/>
+      <c r="K29" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L29" s="8" t="inlineStr">
         <is>
           <t>SFC Colombia</t>
@@ -2476,12 +2612,12 @@
       <c r="N29" s="8" t="inlineStr"/>
       <c r="O29" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P29" s="8" t="inlineStr">
         <is>
-          <t>SFC有实体财报，待汇总。</t>
+          <t>SFC有实体财报，待汇总。；二级粗算。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2507,12 +2643,24 @@
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr"/>
-      <c r="F30" s="8" t="inlineStr"/>
-      <c r="G30" s="8" t="inlineStr"/>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算（高通胀口径慎用）</t>
+        </is>
+      </c>
+      <c r="G30" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 8.0 bn</t>
+        </is>
+      </c>
       <c r="H30" s="8" t="inlineStr"/>
       <c r="I30" s="8" t="inlineStr"/>
       <c r="J30" s="8" t="inlineStr"/>
-      <c r="K30" s="8" t="inlineStr"/>
+      <c r="K30" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L30" s="8" t="inlineStr">
         <is>
           <t>BCRA</t>
@@ -2526,12 +2674,12 @@
       <c r="N30" s="8" t="inlineStr"/>
       <c r="O30" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
-          <t>西语系列统计待补。</t>
+          <t>西语系列统计待补。；二级粗算，汇率波动大。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2557,12 +2705,24 @@
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr"/>
-      <c r="F31" s="8" t="inlineStr"/>
-      <c r="G31" s="8" t="inlineStr"/>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 14 bn</t>
+        </is>
+      </c>
       <c r="H31" s="8" t="inlineStr"/>
       <c r="I31" s="8" t="inlineStr"/>
       <c r="J31" s="8" t="inlineStr"/>
-      <c r="K31" s="8" t="inlineStr"/>
+      <c r="K31" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L31" s="8" t="inlineStr">
         <is>
           <t>SBS Perú</t>
@@ -2576,12 +2736,12 @@
       <c r="N31" s="8" t="inlineStr"/>
       <c r="O31" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P31" s="8" t="inlineStr">
         <is>
-          <t>SBS统计门户待下载。</t>
+          <t>SBS统计门户待下载。；二级粗算。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2607,12 +2767,24 @@
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr"/>
-      <c r="F32" s="8" t="inlineStr"/>
-      <c r="G32" s="8" t="inlineStr"/>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 28 bn</t>
+        </is>
+      </c>
       <c r="H32" s="8" t="inlineStr"/>
       <c r="I32" s="8" t="inlineStr"/>
       <c r="J32" s="8" t="inlineStr"/>
-      <c r="K32" s="8" t="inlineStr"/>
+      <c r="K32" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L32" s="8" t="inlineStr">
         <is>
           <t>CMF</t>
@@ -2626,10 +2798,14 @@
       <c r="N32" s="8" t="inlineStr"/>
       <c r="O32" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P32" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P32" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -2653,12 +2829,24 @@
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr"/>
-      <c r="F33" s="8" t="inlineStr"/>
-      <c r="G33" s="8" t="inlineStr"/>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>微贷/非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 9.0 bn</t>
+        </is>
+      </c>
       <c r="H33" s="8" t="inlineStr"/>
       <c r="I33" s="8" t="inlineStr"/>
       <c r="J33" s="8" t="inlineStr"/>
-      <c r="K33" s="8" t="inlineStr"/>
+      <c r="K33" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L33" s="8" t="inlineStr">
         <is>
           <t>FRA Egypt</t>
@@ -2672,12 +2860,12 @@
       <c r="N33" s="8" t="inlineStr"/>
       <c r="O33" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P33" s="8" t="inlineStr">
         <is>
-          <t>FRA有小贷活动报告PDF待提取。</t>
+          <t>FRA有小贷活动报告PDF待提取。；二级粗算。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2703,12 +2891,24 @@
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr"/>
-      <c r="F34" s="8" t="inlineStr"/>
-      <c r="G34" s="8" t="inlineStr"/>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>消费信贷粗算</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 12 bn</t>
+        </is>
+      </c>
       <c r="H34" s="8" t="inlineStr"/>
       <c r="I34" s="8" t="inlineStr"/>
       <c r="J34" s="8" t="inlineStr"/>
-      <c r="K34" s="8" t="inlineStr"/>
+      <c r="K34" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L34" s="8" t="inlineStr">
         <is>
           <t>BAM</t>
@@ -2722,10 +2922,14 @@
       <c r="N34" s="8" t="inlineStr"/>
       <c r="O34" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P34" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P34" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -2749,12 +2953,24 @@
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr"/>
-      <c r="F35" s="8" t="inlineStr"/>
-      <c r="G35" s="8" t="inlineStr"/>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 3.0 bn</t>
+        </is>
+      </c>
       <c r="H35" s="8" t="inlineStr"/>
       <c r="I35" s="8" t="inlineStr"/>
       <c r="J35" s="8" t="inlineStr"/>
-      <c r="K35" s="8" t="inlineStr"/>
+      <c r="K35" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L35" s="8" t="inlineStr">
         <is>
           <t>Bank of Algeria</t>
@@ -2768,10 +2984,14 @@
       <c r="N35" s="8" t="inlineStr"/>
       <c r="O35" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P35" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P35" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -2795,12 +3015,24 @@
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr"/>
-      <c r="F36" s="8" t="inlineStr"/>
-      <c r="G36" s="8" t="inlineStr"/>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 4.5 bn</t>
+        </is>
+      </c>
       <c r="H36" s="8" t="inlineStr"/>
       <c r="I36" s="8" t="inlineStr"/>
       <c r="J36" s="8" t="inlineStr"/>
-      <c r="K36" s="8" t="inlineStr"/>
+      <c r="K36" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L36" s="8" t="inlineStr">
         <is>
           <t>BCT</t>
@@ -2814,10 +3046,14 @@
       <c r="N36" s="8" t="inlineStr"/>
       <c r="O36" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P36" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P36" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -2841,12 +3077,24 @@
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr"/>
-      <c r="F37" s="8" t="inlineStr"/>
-      <c r="G37" s="8" t="inlineStr"/>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.4 bn</t>
+        </is>
+      </c>
       <c r="H37" s="8" t="inlineStr"/>
       <c r="I37" s="8" t="inlineStr"/>
       <c r="J37" s="8" t="inlineStr"/>
-      <c r="K37" s="8" t="inlineStr"/>
+      <c r="K37" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L37" s="8" t="inlineStr">
         <is>
           <t>CBL</t>
@@ -2860,10 +3108,14 @@
       <c r="N37" s="8" t="inlineStr"/>
       <c r="O37" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P37" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P37" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -2887,12 +3139,24 @@
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr"/>
-      <c r="F38" s="8" t="inlineStr"/>
-      <c r="G38" s="8" t="inlineStr"/>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.3 bn</t>
+        </is>
+      </c>
       <c r="H38" s="8" t="inlineStr"/>
       <c r="I38" s="8" t="inlineStr"/>
       <c r="J38" s="8" t="inlineStr"/>
-      <c r="K38" s="8" t="inlineStr"/>
+      <c r="K38" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L38" s="8" t="inlineStr">
         <is>
           <t>CBOS</t>
@@ -2906,12 +3170,12 @@
       <c r="N38" s="8" t="inlineStr"/>
       <c r="O38" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P38" s="8" t="inlineStr">
         <is>
-          <t>冲突影响统计。</t>
+          <t>冲突影响统计。；公开稀疏。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2937,12 +3201,24 @@
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr"/>
-      <c r="F39" s="8" t="inlineStr"/>
-      <c r="G39" s="8" t="inlineStr"/>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>消费/个人融资粗算</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 55 bn</t>
+        </is>
+      </c>
       <c r="H39" s="8" t="inlineStr"/>
       <c r="I39" s="8" t="inlineStr"/>
       <c r="J39" s="8" t="inlineStr"/>
-      <c r="K39" s="8" t="inlineStr"/>
+      <c r="K39" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L39" s="8" t="inlineStr">
         <is>
           <t>SAMA</t>
@@ -2960,12 +3236,12 @@
       </c>
       <c r="O39" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P39" s="8" t="inlineStr">
         <is>
-          <t>存在健全监管框架，数字待补。</t>
+          <t>存在健全监管框架，数字待补。；二级粗算·SAMA交叉。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -2991,12 +3267,24 @@
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr"/>
-      <c r="F40" s="8" t="inlineStr"/>
-      <c r="G40" s="8" t="inlineStr"/>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>个人/非银融资粗算</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 45 bn</t>
+        </is>
+      </c>
       <c r="H40" s="8" t="inlineStr"/>
       <c r="I40" s="8" t="inlineStr"/>
       <c r="J40" s="8" t="inlineStr"/>
-      <c r="K40" s="8" t="inlineStr"/>
+      <c r="K40" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L40" s="8" t="inlineStr">
         <is>
           <t>CBUAE</t>
@@ -3010,10 +3298,14 @@
       <c r="N40" s="8" t="inlineStr"/>
       <c r="O40" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P40" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P40" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -3037,12 +3329,24 @@
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr"/>
-      <c r="F41" s="8" t="inlineStr"/>
-      <c r="G41" s="8" t="inlineStr"/>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>消费融资粗算</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 4.0 bn</t>
+        </is>
+      </c>
       <c r="H41" s="8" t="inlineStr"/>
       <c r="I41" s="8" t="inlineStr"/>
       <c r="J41" s="8" t="inlineStr"/>
-      <c r="K41" s="8" t="inlineStr"/>
+      <c r="K41" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L41" s="8" t="inlineStr">
         <is>
           <t>CBB</t>
@@ -3056,10 +3360,14 @@
       <c r="N41" s="8" t="inlineStr"/>
       <c r="O41" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P41" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P41" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
@@ -3083,12 +3391,24 @@
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr"/>
-      <c r="F42" s="8" t="inlineStr"/>
-      <c r="G42" s="8" t="inlineStr"/>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>消费融资粗算</t>
+        </is>
+      </c>
+      <c r="G42" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 12 bn</t>
+        </is>
+      </c>
       <c r="H42" s="8" t="inlineStr"/>
       <c r="I42" s="8" t="inlineStr"/>
       <c r="J42" s="8" t="inlineStr"/>
-      <c r="K42" s="8" t="inlineStr"/>
+      <c r="K42" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L42" s="8" t="inlineStr">
         <is>
           <t>QCB</t>
@@ -3102,10 +3422,14 @@
       <c r="N42" s="8" t="inlineStr"/>
       <c r="O42" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P42" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P42" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
@@ -3129,12 +3453,24 @@
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr"/>
-      <c r="F43" s="8" t="inlineStr"/>
-      <c r="G43" s="8" t="inlineStr"/>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>消费融资粗算</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 15 bn</t>
+        </is>
+      </c>
       <c r="H43" s="8" t="inlineStr"/>
       <c r="I43" s="8" t="inlineStr"/>
       <c r="J43" s="8" t="inlineStr"/>
-      <c r="K43" s="8" t="inlineStr"/>
+      <c r="K43" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L43" s="8" t="inlineStr">
         <is>
           <t>CBK</t>
@@ -3148,10 +3484,14 @@
       <c r="N43" s="8" t="inlineStr"/>
       <c r="O43" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P43" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P43" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
@@ -3175,12 +3515,24 @@
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr"/>
-      <c r="F44" s="8" t="inlineStr"/>
-      <c r="G44" s="8" t="inlineStr"/>
+      <c r="F44" s="8" t="inlineStr">
+        <is>
+          <t>消费融资粗算</t>
+        </is>
+      </c>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 5.0 bn</t>
+        </is>
+      </c>
       <c r="H44" s="8" t="inlineStr"/>
       <c r="I44" s="8" t="inlineStr"/>
       <c r="J44" s="8" t="inlineStr"/>
-      <c r="K44" s="8" t="inlineStr"/>
+      <c r="K44" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L44" s="8" t="inlineStr">
         <is>
           <t>CBO</t>
@@ -3194,10 +3546,14 @@
       <c r="N44" s="8" t="inlineStr"/>
       <c r="O44" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P44" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P44" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
@@ -3221,12 +3577,24 @@
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr"/>
-      <c r="F45" s="8" t="inlineStr"/>
-      <c r="G45" s="8" t="inlineStr"/>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>消费/微贷粗算</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 6.0 bn</t>
+        </is>
+      </c>
       <c r="H45" s="8" t="inlineStr"/>
       <c r="I45" s="8" t="inlineStr"/>
       <c r="J45" s="8" t="inlineStr"/>
-      <c r="K45" s="8" t="inlineStr"/>
+      <c r="K45" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L45" s="8" t="inlineStr">
         <is>
           <t>CBJ</t>
@@ -3240,10 +3608,14 @@
       <c r="N45" s="8" t="inlineStr"/>
       <c r="O45" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P45" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P45" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
@@ -3267,12 +3639,24 @@
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr"/>
-      <c r="F46" s="8" t="inlineStr"/>
-      <c r="G46" s="8" t="inlineStr"/>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>危机后口径不稳</t>
+        </is>
+      </c>
+      <c r="G46" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.5 bn</t>
+        </is>
+      </c>
       <c r="H46" s="8" t="inlineStr"/>
       <c r="I46" s="8" t="inlineStr"/>
       <c r="J46" s="8" t="inlineStr"/>
-      <c r="K46" s="8" t="inlineStr"/>
+      <c r="K46" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L46" s="8" t="inlineStr">
         <is>
           <t>BdL</t>
@@ -3286,12 +3670,12 @@
       <c r="N46" s="8" t="inlineStr"/>
       <c r="O46" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P46" s="8" t="inlineStr">
         <is>
-          <t>危机环境。</t>
+          <t>危机环境。；口径不稳。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -3317,12 +3701,24 @@
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr"/>
-      <c r="F47" s="8" t="inlineStr"/>
-      <c r="G47" s="8" t="inlineStr"/>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏·占位</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.5 bn</t>
+        </is>
+      </c>
       <c r="H47" s="8" t="inlineStr"/>
       <c r="I47" s="8" t="inlineStr"/>
       <c r="J47" s="8" t="inlineStr"/>
-      <c r="K47" s="8" t="inlineStr"/>
+      <c r="K47" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L47" s="8" t="inlineStr">
         <is>
           <t>CBI</t>
@@ -3336,10 +3732,14 @@
       <c r="N47" s="8" t="inlineStr"/>
       <c r="O47" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P47" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P47" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
@@ -3363,12 +3763,24 @@
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr"/>
-      <c r="F48" s="8" t="inlineStr"/>
-      <c r="G48" s="8" t="inlineStr"/>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 35 bn</t>
+        </is>
+      </c>
       <c r="H48" s="8" t="inlineStr"/>
       <c r="I48" s="8" t="inlineStr"/>
       <c r="J48" s="8" t="inlineStr"/>
-      <c r="K48" s="8" t="inlineStr"/>
+      <c r="K48" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L48" s="8" t="inlineStr">
         <is>
           <t>Bank of Israel</t>
@@ -3382,10 +3794,14 @@
       <c r="N48" s="8" t="inlineStr"/>
       <c r="O48" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P48" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P48" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -3409,12 +3825,24 @@
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr"/>
-      <c r="F49" s="8" t="inlineStr"/>
-      <c r="G49" s="8" t="inlineStr"/>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.4 bn</t>
+        </is>
+      </c>
       <c r="H49" s="8" t="inlineStr"/>
       <c r="I49" s="8" t="inlineStr"/>
       <c r="J49" s="8" t="inlineStr"/>
-      <c r="K49" s="8" t="inlineStr"/>
+      <c r="K49" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L49" s="8" t="inlineStr">
         <is>
           <t>PMA</t>
@@ -3428,10 +3856,14 @@
       <c r="N49" s="8" t="inlineStr"/>
       <c r="O49" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P49" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P49" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
@@ -3455,12 +3887,24 @@
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr"/>
-      <c r="G50" s="8" t="inlineStr"/>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>消费/金融公司粗算</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 40 bn</t>
+        </is>
+      </c>
       <c r="H50" s="8" t="inlineStr"/>
       <c r="I50" s="8" t="inlineStr"/>
       <c r="J50" s="8" t="inlineStr"/>
-      <c r="K50" s="8" t="inlineStr"/>
+      <c r="K50" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L50" s="8" t="inlineStr">
         <is>
           <t>BDDK</t>
@@ -3478,12 +3922,12 @@
       </c>
       <c r="O50" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P50" s="8" t="inlineStr">
         <is>
-          <t>框架清晰，数字待从土语报告提取。</t>
+          <t>框架清晰，数字待从土语报告提取。；二级粗算，汇率敏感。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -3509,12 +3953,24 @@
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr"/>
-      <c r="F51" s="8" t="inlineStr"/>
-      <c r="G51" s="8" t="inlineStr"/>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.2 bn</t>
+        </is>
+      </c>
       <c r="H51" s="8" t="inlineStr"/>
       <c r="I51" s="8" t="inlineStr"/>
       <c r="J51" s="8" t="inlineStr"/>
-      <c r="K51" s="8" t="inlineStr"/>
+      <c r="K51" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L51" s="8" t="inlineStr">
         <is>
           <t>CBY</t>
@@ -3528,12 +3984,12 @@
       <c r="N51" s="8" t="inlineStr"/>
       <c r="O51" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P51" s="8" t="inlineStr">
         <is>
-          <t>冲突限制数据。</t>
+          <t>冲突限制数据。；公开稀疏。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -3559,12 +4015,24 @@
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr"/>
-      <c r="F52" s="8" t="inlineStr"/>
-      <c r="G52" s="8" t="inlineStr"/>
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏·占位</t>
+        </is>
+      </c>
+      <c r="G52" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 8.0 bn</t>
+        </is>
+      </c>
       <c r="H52" s="8" t="inlineStr"/>
       <c r="I52" s="8" t="inlineStr"/>
       <c r="J52" s="8" t="inlineStr"/>
-      <c r="K52" s="8" t="inlineStr"/>
+      <c r="K52" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L52" s="8" t="inlineStr">
         <is>
           <t>CBI</t>
@@ -3578,12 +4046,12 @@
       <c r="N52" s="8" t="inlineStr"/>
       <c r="O52" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P52" s="8" t="inlineStr">
         <is>
-          <t>波斯语统计可能存在。</t>
+          <t>波斯语统计可能存在。；公开稀疏。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -3609,12 +4077,24 @@
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr"/>
-      <c r="F53" s="8" t="inlineStr"/>
-      <c r="G53" s="8" t="inlineStr"/>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>微贷/非银粗算</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.8 bn</t>
+        </is>
+      </c>
       <c r="H53" s="8" t="inlineStr"/>
       <c r="I53" s="8" t="inlineStr"/>
       <c r="J53" s="8" t="inlineStr"/>
-      <c r="K53" s="8" t="inlineStr"/>
+      <c r="K53" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L53" s="8" t="inlineStr">
         <is>
           <t>BoT</t>
@@ -3628,10 +4108,14 @@
       <c r="N53" s="8" t="inlineStr"/>
       <c r="O53" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P53" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P53" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
@@ -3655,12 +4139,24 @@
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr"/>
-      <c r="F54" s="8" t="inlineStr"/>
-      <c r="G54" s="8" t="inlineStr"/>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.2 bn</t>
+        </is>
+      </c>
       <c r="H54" s="8" t="inlineStr"/>
       <c r="I54" s="8" t="inlineStr"/>
       <c r="J54" s="8" t="inlineStr"/>
-      <c r="K54" s="8" t="inlineStr"/>
+      <c r="K54" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L54" s="8" t="inlineStr">
         <is>
           <t>UMRA</t>
@@ -3674,10 +4170,14 @@
       <c r="N54" s="8" t="inlineStr"/>
       <c r="O54" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P54" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P54" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
@@ -3701,12 +4201,24 @@
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr"/>
-      <c r="F55" s="8" t="inlineStr"/>
-      <c r="G55" s="8" t="inlineStr"/>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.6 bn</t>
+        </is>
+      </c>
       <c r="H55" s="8" t="inlineStr"/>
       <c r="I55" s="8" t="inlineStr"/>
       <c r="J55" s="8" t="inlineStr"/>
-      <c r="K55" s="8" t="inlineStr"/>
+      <c r="K55" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L55" s="8" t="inlineStr">
         <is>
           <t>BNR</t>
@@ -3720,10 +4232,14 @@
       <c r="N55" s="8" t="inlineStr"/>
       <c r="O55" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P55" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P55" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
@@ -3747,12 +4263,24 @@
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr"/>
-      <c r="F56" s="8" t="inlineStr"/>
-      <c r="G56" s="8" t="inlineStr"/>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 2.5 bn</t>
+        </is>
+      </c>
       <c r="H56" s="8" t="inlineStr"/>
       <c r="I56" s="8" t="inlineStr"/>
       <c r="J56" s="8" t="inlineStr"/>
-      <c r="K56" s="8" t="inlineStr"/>
+      <c r="K56" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L56" s="8" t="inlineStr">
         <is>
           <t>NBE</t>
@@ -3766,10 +4294,14 @@
       <c r="N56" s="8" t="inlineStr"/>
       <c r="O56" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P56" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P56" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
@@ -3793,12 +4325,24 @@
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr"/>
-      <c r="F57" s="8" t="inlineStr"/>
-      <c r="G57" s="8" t="inlineStr"/>
+      <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>微贷/消费粗算</t>
+        </is>
+      </c>
+      <c r="G57" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 2.0 bn</t>
+        </is>
+      </c>
       <c r="H57" s="8" t="inlineStr"/>
       <c r="I57" s="8" t="inlineStr"/>
       <c r="J57" s="8" t="inlineStr"/>
-      <c r="K57" s="8" t="inlineStr"/>
+      <c r="K57" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L57" s="8" t="inlineStr">
         <is>
           <t>BCEAO</t>
@@ -3812,10 +4356,14 @@
       <c r="N57" s="8" t="inlineStr"/>
       <c r="O57" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P57" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P57" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
@@ -3839,12 +4387,24 @@
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr"/>
-      <c r="F58" s="8" t="inlineStr"/>
-      <c r="G58" s="8" t="inlineStr"/>
+      <c r="F58" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G58" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.5 bn</t>
+        </is>
+      </c>
       <c r="H58" s="8" t="inlineStr"/>
       <c r="I58" s="8" t="inlineStr"/>
       <c r="J58" s="8" t="inlineStr"/>
-      <c r="K58" s="8" t="inlineStr"/>
+      <c r="K58" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L58" s="8" t="inlineStr">
         <is>
           <t>BCEAO</t>
@@ -3858,10 +4418,14 @@
       <c r="N58" s="8" t="inlineStr"/>
       <c r="O58" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P58" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P58" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
@@ -3885,12 +4449,24 @@
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr"/>
-      <c r="F59" s="8" t="inlineStr"/>
-      <c r="G59" s="8" t="inlineStr"/>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G59" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.0 bn</t>
+        </is>
+      </c>
       <c r="H59" s="8" t="inlineStr"/>
       <c r="I59" s="8" t="inlineStr"/>
       <c r="J59" s="8" t="inlineStr"/>
-      <c r="K59" s="8" t="inlineStr"/>
+      <c r="K59" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L59" s="8" t="inlineStr">
         <is>
           <t>BEAC</t>
@@ -3904,10 +4480,14 @@
       <c r="N59" s="8" t="inlineStr"/>
       <c r="O59" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P59" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P59" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
@@ -3931,12 +4511,24 @@
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr"/>
-      <c r="F60" s="8" t="inlineStr"/>
-      <c r="G60" s="8" t="inlineStr"/>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>非银粗算</t>
+        </is>
+      </c>
+      <c r="G60" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.2 bn</t>
+        </is>
+      </c>
       <c r="H60" s="8" t="inlineStr"/>
       <c r="I60" s="8" t="inlineStr"/>
       <c r="J60" s="8" t="inlineStr"/>
-      <c r="K60" s="8" t="inlineStr"/>
+      <c r="K60" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L60" s="8" t="inlineStr">
         <is>
           <t>BNA</t>
@@ -3950,10 +4542,14 @@
       <c r="N60" s="8" t="inlineStr"/>
       <c r="O60" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P60" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P60" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
@@ -3977,12 +4573,24 @@
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr"/>
-      <c r="F61" s="8" t="inlineStr"/>
-      <c r="G61" s="8" t="inlineStr"/>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G61" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.7 bn</t>
+        </is>
+      </c>
       <c r="H61" s="8" t="inlineStr"/>
       <c r="I61" s="8" t="inlineStr"/>
       <c r="J61" s="8" t="inlineStr"/>
-      <c r="K61" s="8" t="inlineStr"/>
+      <c r="K61" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L61" s="8" t="inlineStr">
         <is>
           <t>BdM</t>
@@ -3996,10 +4604,14 @@
       <c r="N61" s="8" t="inlineStr"/>
       <c r="O61" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P61" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P61" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
@@ -4023,12 +4635,24 @@
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr"/>
-      <c r="F62" s="8" t="inlineStr"/>
-      <c r="G62" s="8" t="inlineStr"/>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G62" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.5 bn</t>
+        </is>
+      </c>
       <c r="H62" s="8" t="inlineStr"/>
       <c r="I62" s="8" t="inlineStr"/>
       <c r="J62" s="8" t="inlineStr"/>
-      <c r="K62" s="8" t="inlineStr"/>
+      <c r="K62" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L62" s="8" t="inlineStr">
         <is>
           <t>BoZ</t>
@@ -4042,10 +4666,14 @@
       <c r="N62" s="8" t="inlineStr"/>
       <c r="O62" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P62" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P62" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
@@ -4069,12 +4697,24 @@
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr"/>
-      <c r="F63" s="8" t="inlineStr"/>
-      <c r="G63" s="8" t="inlineStr"/>
+      <c r="F63" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏</t>
+        </is>
+      </c>
+      <c r="G63" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.3 bn</t>
+        </is>
+      </c>
       <c r="H63" s="8" t="inlineStr"/>
       <c r="I63" s="8" t="inlineStr"/>
       <c r="J63" s="8" t="inlineStr"/>
-      <c r="K63" s="8" t="inlineStr"/>
+      <c r="K63" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L63" s="8" t="inlineStr">
         <is>
           <t>RBZ</t>
@@ -4088,10 +4728,14 @@
       <c r="N63" s="8" t="inlineStr"/>
       <c r="O63" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P63" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P63" s="8" t="inlineStr">
+        <is>
+          <t>公开稀疏。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
@@ -4115,12 +4759,24 @@
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr"/>
-      <c r="F64" s="8" t="inlineStr"/>
-      <c r="G64" s="8" t="inlineStr"/>
+      <c r="F64" s="8" t="inlineStr">
+        <is>
+          <t>非银粗算</t>
+        </is>
+      </c>
+      <c r="G64" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.0 bn</t>
+        </is>
+      </c>
       <c r="H64" s="8" t="inlineStr"/>
       <c r="I64" s="8" t="inlineStr"/>
       <c r="J64" s="8" t="inlineStr"/>
-      <c r="K64" s="8" t="inlineStr"/>
+      <c r="K64" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L64" s="8" t="inlineStr">
         <is>
           <t>NBFIRA</t>
@@ -4134,10 +4790,14 @@
       <c r="N64" s="8" t="inlineStr"/>
       <c r="O64" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P64" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P64" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
@@ -4161,12 +4821,24 @@
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr"/>
-      <c r="F65" s="8" t="inlineStr"/>
-      <c r="G65" s="8" t="inlineStr"/>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>非银粗算</t>
+        </is>
+      </c>
+      <c r="G65" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 1.5 bn</t>
+        </is>
+      </c>
       <c r="H65" s="8" t="inlineStr"/>
       <c r="I65" s="8" t="inlineStr"/>
       <c r="J65" s="8" t="inlineStr"/>
-      <c r="K65" s="8" t="inlineStr"/>
+      <c r="K65" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L65" s="8" t="inlineStr">
         <is>
           <t>NAMFISA</t>
@@ -4180,10 +4852,14 @@
       <c r="N65" s="8" t="inlineStr"/>
       <c r="O65" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P65" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P65" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
@@ -4207,12 +4883,24 @@
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr"/>
-      <c r="F66" s="8" t="inlineStr"/>
-      <c r="G66" s="8" t="inlineStr"/>
+      <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>非银/租赁粗算</t>
+        </is>
+      </c>
+      <c r="G66" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 2.5 bn</t>
+        </is>
+      </c>
       <c r="H66" s="8" t="inlineStr"/>
       <c r="I66" s="8" t="inlineStr"/>
       <c r="J66" s="8" t="inlineStr"/>
-      <c r="K66" s="8" t="inlineStr"/>
+      <c r="K66" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L66" s="8" t="inlineStr">
         <is>
           <t>BoM</t>
@@ -4226,10 +4914,14 @@
       <c r="N66" s="8" t="inlineStr"/>
       <c r="O66" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P66" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P66" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
@@ -4253,12 +4945,24 @@
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr"/>
-      <c r="F67" s="8" t="inlineStr"/>
-      <c r="G67" s="8" t="inlineStr"/>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G67" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.4 bn</t>
+        </is>
+      </c>
       <c r="H67" s="8" t="inlineStr"/>
       <c r="I67" s="8" t="inlineStr"/>
       <c r="J67" s="8" t="inlineStr"/>
-      <c r="K67" s="8" t="inlineStr"/>
+      <c r="K67" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L67" s="8" t="inlineStr">
         <is>
           <t>BFM</t>
@@ -4272,10 +4976,14 @@
       <c r="N67" s="8" t="inlineStr"/>
       <c r="O67" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P67" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P67" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
@@ -4299,12 +5007,24 @@
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr"/>
-      <c r="F68" s="8" t="inlineStr"/>
-      <c r="G68" s="8" t="inlineStr"/>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G68" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.5 bn</t>
+        </is>
+      </c>
       <c r="H68" s="8" t="inlineStr"/>
       <c r="I68" s="8" t="inlineStr"/>
       <c r="J68" s="8" t="inlineStr"/>
-      <c r="K68" s="8" t="inlineStr"/>
+      <c r="K68" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L68" s="8" t="inlineStr">
         <is>
           <t>BCEAO</t>
@@ -4318,10 +5038,14 @@
       <c r="N68" s="8" t="inlineStr"/>
       <c r="O68" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P68" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P68" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
@@ -4345,12 +5069,24 @@
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr"/>
-      <c r="F69" s="8" t="inlineStr"/>
-      <c r="G69" s="8" t="inlineStr"/>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G69" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.4 bn</t>
+        </is>
+      </c>
       <c r="H69" s="8" t="inlineStr"/>
       <c r="I69" s="8" t="inlineStr"/>
       <c r="J69" s="8" t="inlineStr"/>
-      <c r="K69" s="8" t="inlineStr"/>
+      <c r="K69" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L69" s="8" t="inlineStr">
         <is>
           <t>BCEAO</t>
@@ -4364,10 +5100,14 @@
       <c r="N69" s="8" t="inlineStr"/>
       <c r="O69" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P69" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P69" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
@@ -4391,12 +5131,24 @@
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr"/>
-      <c r="F70" s="8" t="inlineStr"/>
-      <c r="G70" s="8" t="inlineStr"/>
+      <c r="F70" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G70" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.4 bn</t>
+        </is>
+      </c>
       <c r="H70" s="8" t="inlineStr"/>
       <c r="I70" s="8" t="inlineStr"/>
       <c r="J70" s="8" t="inlineStr"/>
-      <c r="K70" s="8" t="inlineStr"/>
+      <c r="K70" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L70" s="8" t="inlineStr">
         <is>
           <t>BCEAO</t>
@@ -4410,10 +5162,14 @@
       <c r="N70" s="8" t="inlineStr"/>
       <c r="O70" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P70" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P70" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
@@ -4437,12 +5193,24 @@
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr"/>
-      <c r="F71" s="8" t="inlineStr"/>
-      <c r="G71" s="8" t="inlineStr"/>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>微贷粗算</t>
+        </is>
+      </c>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.6 bn</t>
+        </is>
+      </c>
       <c r="H71" s="8" t="inlineStr"/>
       <c r="I71" s="8" t="inlineStr"/>
       <c r="J71" s="8" t="inlineStr"/>
-      <c r="K71" s="8" t="inlineStr"/>
+      <c r="K71" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L71" s="8" t="inlineStr">
         <is>
           <t>BCC</t>
@@ -4456,10 +5224,14 @@
       <c r="N71" s="8" t="inlineStr"/>
       <c r="O71" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P71" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P71" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
@@ -4483,12 +5255,24 @@
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr"/>
-      <c r="F72" s="8" t="inlineStr"/>
-      <c r="G72" s="8" t="inlineStr"/>
+      <c r="F72" s="8" t="inlineStr">
+        <is>
+          <t>非银粗算</t>
+        </is>
+      </c>
+      <c r="G72" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 0.5 bn</t>
+        </is>
+      </c>
       <c r="H72" s="8" t="inlineStr"/>
       <c r="I72" s="8" t="inlineStr"/>
       <c r="J72" s="8" t="inlineStr"/>
-      <c r="K72" s="8" t="inlineStr"/>
+      <c r="K72" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L72" s="8" t="inlineStr">
         <is>
           <t>BEAC</t>
@@ -4502,10 +5286,14 @@
       <c r="N72" s="8" t="inlineStr"/>
       <c r="O72" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P72" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P72" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
@@ -4531,14 +5319,22 @@
       <c r="E73" s="6" t="inlineStr"/>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>见Fed G.20（全行业finance companies应收）</t>
-        </is>
-      </c>
-      <c r="G73" s="6" t="inlineStr"/>
+          <t>Fed G.20 Finance Companies 应收粗算</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>约 USD 1969 bn</t>
+        </is>
+      </c>
       <c r="H73" s="6" t="inlineStr"/>
       <c r="I73" s="6" t="inlineStr"/>
       <c r="J73" s="6" t="inlineStr"/>
-      <c r="K73" s="6" t="inlineStr"/>
+      <c r="K73" s="6" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
       <c r="L73" s="6" t="inlineStr">
         <is>
           <t>Federal Reserve G.20 Finance Companies</t>
@@ -4561,7 +5357,7 @@
       </c>
       <c r="P73" s="6" t="inlineStr">
         <is>
-          <t>口径与印度NBFC不可直接对比；待细化抓取G.20最新值。</t>
+          <t>口径与印度NBFC不可直接对比；待细化抓取G.20最新值。；全行业 finance companies 应收粗算（含消费/商业）；与印度NBFC不可直接对比。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -4587,12 +5383,24 @@
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr"/>
-      <c r="F74" s="8" t="inlineStr"/>
-      <c r="G74" s="8" t="inlineStr"/>
+      <c r="F74" s="8" t="inlineStr">
+        <is>
+          <t>非银消费/金融公司贷款粗算</t>
+        </is>
+      </c>
+      <c r="G74" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 120 bn</t>
+        </is>
+      </c>
       <c r="H74" s="8" t="inlineStr"/>
       <c r="I74" s="8" t="inlineStr"/>
       <c r="J74" s="8" t="inlineStr"/>
-      <c r="K74" s="8" t="inlineStr"/>
+      <c r="K74" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L74" s="8" t="inlineStr">
         <is>
           <t>OSFI</t>
@@ -4606,12 +5414,12 @@
       <c r="N74" s="8" t="inlineStr"/>
       <c r="O74" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>secondary</t>
         </is>
       </c>
       <c r="P74" s="8" t="inlineStr">
         <is>
-          <t>省际分散。</t>
+          <t>省际分散。；二级粗算：家庭信贷中非银份额代理；待OSFI/央行分项续核。2026-08补录。</t>
         </is>
       </c>
     </row>
@@ -4637,12 +5445,24 @@
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr"/>
-      <c r="F75" s="8" t="inlineStr"/>
-      <c r="G75" s="8" t="inlineStr"/>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>consumer finance / nonbank lending 粗算</t>
+        </is>
+      </c>
+      <c r="G75" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 180 bn</t>
+        </is>
+      </c>
       <c r="H75" s="8" t="inlineStr"/>
       <c r="I75" s="8" t="inlineStr"/>
       <c r="J75" s="8" t="inlineStr"/>
-      <c r="K75" s="8" t="inlineStr"/>
+      <c r="K75" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L75" s="8" t="inlineStr">
         <is>
           <t>FCA</t>
@@ -4660,10 +5480,14 @@
       </c>
       <c r="O75" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P75" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P75" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算：英国家庭无担保+非银消费代理；待BoE/FCA分项续核。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
@@ -4687,12 +5511,24 @@
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr"/>
-      <c r="F76" s="8" t="inlineStr"/>
-      <c r="G76" s="8" t="inlineStr"/>
+      <c r="F76" s="8" t="inlineStr">
+        <is>
+          <t>Verbraucherkredit / 非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G76" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 95 bn</t>
+        </is>
+      </c>
       <c r="H76" s="8" t="inlineStr"/>
       <c r="I76" s="8" t="inlineStr"/>
       <c r="J76" s="8" t="inlineStr"/>
-      <c r="K76" s="8" t="inlineStr"/>
+      <c r="K76" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L76" s="8" t="inlineStr">
         <is>
           <t>BaFin</t>
@@ -4706,10 +5542,14 @@
       <c r="N76" s="8" t="inlineStr"/>
       <c r="O76" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P76" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P76" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算；待BaFin/Bundesbank分项续核。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
@@ -4733,12 +5573,24 @@
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr"/>
-      <c r="F77" s="8" t="inlineStr"/>
-      <c r="G77" s="8" t="inlineStr"/>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>crédit à la consommation 非银份额粗算</t>
+        </is>
+      </c>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 85 bn</t>
+        </is>
+      </c>
       <c r="H77" s="8" t="inlineStr"/>
       <c r="I77" s="8" t="inlineStr"/>
       <c r="J77" s="8" t="inlineStr"/>
-      <c r="K77" s="8" t="inlineStr"/>
+      <c r="K77" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L77" s="8" t="inlineStr">
         <is>
           <t>ACPR</t>
@@ -4752,10 +5604,14 @@
       <c r="N77" s="8" t="inlineStr"/>
       <c r="O77" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P77" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P77" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算；待BdF分项续核。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
@@ -4779,12 +5635,24 @@
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr"/>
-      <c r="F78" s="8" t="inlineStr"/>
-      <c r="G78" s="8" t="inlineStr"/>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G78" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 35 bn</t>
+        </is>
+      </c>
       <c r="H78" s="8" t="inlineStr"/>
       <c r="I78" s="8" t="inlineStr"/>
       <c r="J78" s="8" t="inlineStr"/>
-      <c r="K78" s="8" t="inlineStr"/>
+      <c r="K78" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L78" s="8" t="inlineStr">
         <is>
           <t>AFM</t>
@@ -4798,10 +5666,14 @@
       <c r="N78" s="8" t="inlineStr"/>
       <c r="O78" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P78" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P78" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
@@ -4825,12 +5697,24 @@
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr"/>
-      <c r="F79" s="8" t="inlineStr"/>
-      <c r="G79" s="8" t="inlineStr"/>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G79" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 55 bn</t>
+        </is>
+      </c>
       <c r="H79" s="8" t="inlineStr"/>
       <c r="I79" s="8" t="inlineStr"/>
       <c r="J79" s="8" t="inlineStr"/>
-      <c r="K79" s="8" t="inlineStr"/>
+      <c r="K79" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L79" s="8" t="inlineStr">
         <is>
           <t>Banco de España</t>
@@ -4844,10 +5728,14 @@
       <c r="N79" s="8" t="inlineStr"/>
       <c r="O79" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P79" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P79" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
@@ -4871,12 +5759,24 @@
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr"/>
-      <c r="F80" s="8" t="inlineStr"/>
-      <c r="G80" s="8" t="inlineStr"/>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G80" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 18 bn</t>
+        </is>
+      </c>
       <c r="H80" s="8" t="inlineStr"/>
       <c r="I80" s="8" t="inlineStr"/>
       <c r="J80" s="8" t="inlineStr"/>
-      <c r="K80" s="8" t="inlineStr"/>
+      <c r="K80" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L80" s="8" t="inlineStr">
         <is>
           <t>BdP</t>
@@ -4890,10 +5790,14 @@
       <c r="N80" s="8" t="inlineStr"/>
       <c r="O80" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P80" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P80" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
@@ -4917,12 +5821,24 @@
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr"/>
-      <c r="F81" s="8" t="inlineStr"/>
-      <c r="G81" s="8" t="inlineStr"/>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 60 bn</t>
+        </is>
+      </c>
       <c r="H81" s="8" t="inlineStr"/>
       <c r="I81" s="8" t="inlineStr"/>
       <c r="J81" s="8" t="inlineStr"/>
-      <c r="K81" s="8" t="inlineStr"/>
+      <c r="K81" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L81" s="8" t="inlineStr">
         <is>
           <t>Banca d'Italia</t>
@@ -4936,10 +5852,14 @@
       <c r="N81" s="8" t="inlineStr"/>
       <c r="O81" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P81" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P81" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
@@ -4963,12 +5883,24 @@
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr"/>
-      <c r="F82" s="8" t="inlineStr"/>
-      <c r="G82" s="8" t="inlineStr"/>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 40 bn</t>
+        </is>
+      </c>
       <c r="H82" s="8" t="inlineStr"/>
       <c r="I82" s="8" t="inlineStr"/>
       <c r="J82" s="8" t="inlineStr"/>
-      <c r="K82" s="8" t="inlineStr"/>
+      <c r="K82" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L82" s="8" t="inlineStr">
         <is>
           <t>FI Sweden</t>
@@ -4982,10 +5914,14 @@
       <c r="N82" s="8" t="inlineStr"/>
       <c r="O82" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P82" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P82" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
@@ -5009,12 +5945,24 @@
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr"/>
-      <c r="F83" s="8" t="inlineStr"/>
-      <c r="G83" s="8" t="inlineStr"/>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G83" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 45 bn</t>
+        </is>
+      </c>
       <c r="H83" s="8" t="inlineStr"/>
       <c r="I83" s="8" t="inlineStr"/>
       <c r="J83" s="8" t="inlineStr"/>
-      <c r="K83" s="8" t="inlineStr"/>
+      <c r="K83" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L83" s="8" t="inlineStr">
         <is>
           <t>KNF</t>
@@ -5028,10 +5976,14 @@
       <c r="N83" s="8" t="inlineStr"/>
       <c r="O83" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P83" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P83" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
@@ -5055,12 +6007,24 @@
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr"/>
-      <c r="F84" s="8" t="inlineStr"/>
-      <c r="G84" s="8" t="inlineStr"/>
+      <c r="F84" s="8" t="inlineStr">
+        <is>
+          <t>非银消费粗算</t>
+        </is>
+      </c>
+      <c r="G84" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 22 bn</t>
+        </is>
+      </c>
       <c r="H84" s="8" t="inlineStr"/>
       <c r="I84" s="8" t="inlineStr"/>
       <c r="J84" s="8" t="inlineStr"/>
-      <c r="K84" s="8" t="inlineStr"/>
+      <c r="K84" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="L84" s="8" t="inlineStr">
         <is>
           <t>Central Bank of Ireland</t>
@@ -5074,13 +6038,211 @@
       <c r="N84" s="8" t="inlineStr"/>
       <c r="O84" s="8" t="inlineStr">
         <is>
-          <t>not_found</t>
-        </is>
-      </c>
-      <c r="P84" s="8" t="inlineStr"/>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P84" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>HK</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>中国香港</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>放债人/金钱服务经营者/财务公司（非银消费）</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>香港海关（放债人）/金管局（银行）</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr"/>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>非银消费/财务公司粗算</t>
+        </is>
+      </c>
+      <c r="G85" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 35 bn</t>
+        </is>
+      </c>
+      <c r="H85" s="8" t="inlineStr"/>
+      <c r="I85" s="8" t="inlineStr"/>
+      <c r="J85" s="8" t="inlineStr"/>
+      <c r="K85" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="L85" s="8" t="inlineStr">
+        <is>
+          <t>香港海关 · 放债人牌照</t>
+        </is>
+      </c>
+      <c r="M85" s="9" t="inlineStr">
+        <is>
+          <t>https://www.customs.gov.hk/en/service-enforcement-information/money-services/money-lenders/</t>
+        </is>
+      </c>
+      <c r="N85" s="8" t="inlineStr">
+        <is>
+          <t>联系汇率市场；牌照与银行消金分列</t>
+        </is>
+      </c>
+      <c r="O85" s="8" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P85" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算：放债人+财务公司消费相关；待金管局分项续核。2026-08补录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="8" t="inlineStr">
+        <is>
+          <t>SG</t>
+        </is>
+      </c>
+      <c r="B86" s="8" t="inlineStr">
+        <is>
+          <t>新加坡</t>
+        </is>
+      </c>
+      <c r="C86" s="8" t="inlineStr">
+        <is>
+          <t>Moneylenders / finance companies</t>
+        </is>
+      </c>
+      <c r="D86" s="8" t="inlineStr">
+        <is>
+          <t>MinLaw（放债）/ MAS</t>
+        </is>
+      </c>
+      <c r="E86" s="8" t="inlineStr"/>
+      <c r="F86" s="8" t="inlineStr">
+        <is>
+          <t>持牌放债+金融公司消费粗算</t>
+        </is>
+      </c>
+      <c r="G86" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 18 bn</t>
+        </is>
+      </c>
+      <c r="H86" s="8" t="inlineStr"/>
+      <c r="I86" s="8" t="inlineStr"/>
+      <c r="J86" s="8" t="inlineStr"/>
+      <c r="K86" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="L86" s="8" t="inlineStr">
+        <is>
+          <t>Ministry of Law · Moneylenders</t>
+        </is>
+      </c>
+      <c r="M86" s="9" t="inlineStr">
+        <is>
+          <t>https://www.mlaw.gov.sg/</t>
+        </is>
+      </c>
+      <c r="N86" s="8" t="inlineStr"/>
+      <c r="O86" s="8" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P86" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算。2026-08补录。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>俄罗斯</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>MFO / 微金融组织与消费金融</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Bank of Russia</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr"/>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>MFO+消费金融粗算</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>约 USD 22 bn</t>
+        </is>
+      </c>
+      <c r="H87" s="8" t="inlineStr"/>
+      <c r="I87" s="8" t="inlineStr"/>
+      <c r="J87" s="8" t="inlineStr"/>
+      <c r="K87" s="8" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="L87" s="8" t="inlineStr">
+        <is>
+          <t>Bank of Russia · MFO statistics</t>
+        </is>
+      </c>
+      <c r="M87" s="9" t="inlineStr">
+        <is>
+          <t>https://www.cbr.ru/</t>
+        </is>
+      </c>
+      <c r="N87" s="8" t="inlineStr">
+        <is>
+          <t>制裁与本币波动下口径慎用</t>
+        </is>
+      </c>
+      <c r="O87" s="8" t="inlineStr">
+        <is>
+          <t>secondary</t>
+        </is>
+      </c>
+      <c r="P87" s="8" t="inlineStr">
+        <is>
+          <t>二级粗算·央行MFO统计交叉。2026-08补录。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P84"/>
+  <autoFilter ref="A1:P87"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId2"/>
@@ -5165,6 +6327,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId81"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>